<commit_message>
Defect Register v0.5: DEF-014, DEF-015, DEF-017 closed, DEF-020 added; Technical Debt Register v0.3: TD-004 repaid, TD-005 to TD-008 added
DEF-014, DEF-015 and DEF-017 closed on the test (PR #102) and staging (PR #111) evidence, with R. van der Merwe's closure text; residual: production has no cluster yet. DEF-020 (S2, P1, Closed): the staging MONGODB_URI named no database, so the application used the default test database until 16:12:28 UTC on 15/10/2026; fixed before the load run and smoke test (PR #111). TD-004 repaid on the test and staging clusters. New: TD-005 (AC-FR-1.3, a rejected operation is not recorded), TD-006 (no unit test asserts a reject without a reason is refused), TD-007 (the OpenAPI tests do not parse the YAML), TD-008 (the 8 integration cases never run in CI, C. Burger). v0.2 moved unchanged to Outdated/.
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.5.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c906530d9ff38bc/Desktop/SEN381/Ticketing-System/docs/quality/Defect Register/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="11_1E414E22D62B1D240B6507ADAE6B1F6F79FB2D4F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B5066CA-98E1-4E5B-B343-4A6B25D85A11}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="11_1E414E22D62B1D240B6507ADAE6B1F6F79FB2D4F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D87FCE16-DF3F-4584-8348-859197FAF3DB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Defect Register" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$30</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="172">
   <si>
     <t>Defect Register</t>
   </si>
@@ -470,42 +470,9 @@
     <t>Not release-blocking (S3). Residual: the cause of three test failures is unknown, and they cannot be ruled out as a real fault.</t>
   </si>
   <si>
-    <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.5 (15/10/2026). Adds DEF-019 (two test titles cite the wrong requirement), raised by E. Lindsay. DEF-006, DEF-014, DEF-015 and DEF-017 updated with the test-cluster index provisioning and duplicate-refusal results (PR #98, PR #102); their status is unchanged (Open) and staging is pending, updated by E. Lindsay. DEF-001 to DEF-005, DEF-007 to DEF-013, DEF-016 and DEF-018 unchanged. Version 0.4 (14/10/2026). Adds DEF-018 (an unexplained npm test failure in the PR #98 build: 3 failures, test names not captured), raised by R. van der Merwe. DEF-001 to DEF-017 unchanged. Version 0.3 (12/10/2026). Adds DEF-017 (the unique index on users.email is absent on the test cluster; FR-1.1 relies on it alone), raised by E. Lindsay; DEF-014 and DEF-015 cell E updated with the observed index absence from the test-cluster listing. DEF-001 to DEF-016 otherwise unchanged. Version 0.2 (12/10/2026). Adds DEF-005 to DEF-016: DEF-007 to DEF-010, DEF-014, and DEF-015 from M3 integration testing (R. van der Merwe); DEF-005, DEF-006, DEF-011 to DEF-013, and DEF-016 raised by E. Lindsay. DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
-  </si>
-  <si>
     <t>The test cluster database is not dropped per run, contradicting DEC-003's test-environment row and our own smoke script docstring. Update v0.5: the test cluster's civicconnect database was dropped once, by R. van der Merwe through the Atlas UI at 15:55 UTC on 14/10/2026, before the index provisioning runs (docs/evidence/M3-indexes/index_provisioning_test_run1.txt, note of 15/10/2026). A one-off drop, not a per-run drop: the defect is unchanged. Runs since then have added synthetic data again (the L2 to L4 checks on 14/10/2026; the E2E run at v3.0-M3-rc on 15/10/2026).</t>
   </si>
   <si>
-    <t>Test cluster: fixed by TD-004's provisioning step (scripts/atlas/provision-indexes.js, PR #98; DEC-003 v0.3 deployment step 5). Runs 1 and 2 on 14/10/2026 created and confirmed actorId_1_idempotencyKey_1 (unique, partial: string keys only). Staging: pending; the step runs before the first staging deploy (DEC-003 v0.4).</t>
-  </si>
-  <si>
-    <t>PR #98 (script and tests); PR #102 (test-cluster runs 1 and 2, and the L2 to L4 checks)</t>
-  </si>
-  <si>
-    <t>Test cluster: L2, a duplicate (actorId, idempotencyKey) refused by the database with 11000 naming actorId_1_idempotencyKey_1, and L2c, the partial-filter control (docs/evidence/M3-indexes/index_duplicate_refusal_test_2026-10-14.txt). Before: the duplicate accepted (docs/evidence/M3_API_Negative_Verification.txt) and the index absent (docs/evidence/M3-indexes/index_check_L1_test_2026-10-13.txt). Staging: pending.</t>
-  </si>
-  <si>
-    <t>Open. S2: release only with the limitation recorded, unless fixed first. Residual: on the test cluster the index now exists and refuses a duplicate key. On staging it is pending until the staging provisioning run is recorded; production is unverified. Not shown: a real concurrent race, or how the API reports an 11000 error.</t>
-  </si>
-  <si>
-    <t>Test cluster: fixed by TD-004's provisioning step (scripts/atlas/provision-indexes.js, PR #98; DEC-003 v0.3 deployment step 5). Runs 1 and 2 on 14/10/2026 created and confirmed requestId_1_requestVersion_1 (unique). Staging: pending; the step runs before the first staging deploy (DEC-003 v0.4).</t>
-  </si>
-  <si>
-    <t>Test cluster: L3, a duplicate (requestId, requestVersion) refused by the database with 11000 naming requestId_1_requestVersion_1 (docs/evidence/M3-indexes/index_duplicate_refusal_test_2026-10-14.txt). Before: the duplicate accepted (docs/evidence/M3_API_Negative_Verification.txt) and the index absent (docs/evidence/M3-indexes/index_check_L1_test_2026-10-13.txt). Staging: pending.</t>
-  </si>
-  <si>
-    <t>Open. S2: release only with the limitation recorded, unless fixed first. Residual: on the test cluster the index now exists and refuses a second entry for the same version. On staging it is pending until the staging provisioning run is recorded; production is unverified. Not shown: two transitions actually racing.</t>
-  </si>
-  <si>
-    <t>Test cluster: fixed by TD-004's provisioning step (scripts/atlas/provision-indexes.js, PR #98; DEC-003 v0.3 deployment step 5). Runs 1 and 2 on 14/10/2026 created and confirmed email_1 (unique). Staging: pending; the step runs before the first staging deploy (DEC-003 v0.4). Still to decide with the staging fix: whether scripts/admin/create-user.js should also check for an existing email before inserting.</t>
-  </si>
-  <si>
-    <t>Test cluster: L4, a second user with the same email refused by the database with 11000 naming email_1 (docs/evidence/M3-indexes/index_duplicate_refusal_test_2026-10-14.txt). L4 inserts through the User model, which lowercases and trims email, so it shows an identical stored email is refused, not what happens to a write that bypasses the model. Before: email_1 absent (docs/evidence/M3-indexes/index_check_L1_test_2026-10-13.txt). Staging: pending.</t>
-  </si>
-  <si>
-    <t>Open. S2: release only with the limitation recorded, unless fixed first. Residual: on the test cluster the database now refuses a duplicate email. On staging it is pending until the staging provisioning run is recorded; production is unverified.</t>
-  </si>
-  <si>
     <t>DEF-019</t>
   </si>
   <si>
@@ -528,6 +495,63 @@
   </si>
   <si>
     <t>Not release-blocking (S3). Residual: two test titles carry wrong citations until corrected; the RTM records the correct ones.</t>
+  </si>
+  <si>
+    <t>M3 brief §12: "Maintain a simple defect record: defect -&gt; severity/impact -&gt; status -&gt; fix -&gt; regression evidence where corrected." §15: "Known defects | Open/closed | Business impact | Block or residual risk". Each row has a stable DEF identifier the RTM Defect/Status column can cite. Identifiers are never reused or renumbered; a closed defect stays in the register. | Version 0.5 (15/10/2026). Adds DEF-019 (two test titles cite the wrong requirement), raised by E. Lindsay, and DEF-020 (the staging MONGODB_URI named no database, so the application used the default test database), raised by R. van der Merwe. Closes DEF-014, DEF-015 and DEF-017: their unique indexes were provisioned and confirmed on the test cluster (PR #102) and the staging cluster (PR #111); closure text by R. van der Merwe, entered by E. Lindsay. DEF-006 records the one-off drop of the test database on 14/10/2026. DEF-001 to DEF-005, DEF-007 to DEF-013, DEF-016 and DEF-018 unchanged. Version 0.4 (14/10/2026). Adds DEF-018 (an unexplained npm test failure in the PR #98 build: 3 failures, test names not captured), raised by R. van der Merwe. DEF-001 to DEF-017 unchanged. Version 0.3 (12/10/2026). Adds DEF-017 (the unique index on users.email is absent on the test cluster; FR-1.1 relies on it alone), raised by E. Lindsay; DEF-014 and DEF-015 cell E updated with the observed index absence from the test-cluster listing. DEF-001 to DEF-016 otherwise unchanged. Version 0.2 (12/10/2026). Adds DEF-005 to DEF-016: DEF-007 to DEF-010, DEF-014, and DEF-015 from M3 integration testing (R. van der Merwe); DEF-005, DEF-006, DEF-011 to DEF-013, and DEF-016 raised by E. Lindsay. DEF-001 to DEF-004 unchanged. Version 0.1 (11/10/2026). Register created with DEF-001 to DEF-004.</t>
+  </si>
+  <si>
+    <t>The unique index actorId_1_idempotencyKey_1 was built by scripts/atlas/provision-indexes.js under the temporary civicconnect-temp-provisioner user (TD-004; DEC-003 v0.4 step 5): on the test cluster on 2026-10-14 and on the staging cluster on 2026-10-15.</t>
+  </si>
+  <si>
+    <t>PR #98 (script); PR #102 (test-cluster evidence); PR #111 (staging evidence)</t>
+  </si>
+  <si>
+    <t>docs/evidence/M3-indexes/index_duplicate_refusal_test_2026-10-14.txt, L2: a duplicate (actorId, idempotencyKey) refused with 11000 naming the index, and L2c: entries without a key still accepted. On staging the index is listed as present and unique: docs/evidence/M3-indexes/index_provisioning_staging_run1.txt and _run2.txt (PR #111): RESULT PASS 21 of 21 on the staging cluster, 2026-10-15. Duplicate refusal itself was exercised on the test cluster only.</t>
+  </si>
+  <si>
+    <t>Closed on the test and staging clusters. Residual: production has no cluster yet; DEC-003 v0.4 step 5 must run there before its first deploy.</t>
+  </si>
+  <si>
+    <t>The unique index requestId_1_requestVersion_1 was built by scripts/atlas/provision-indexes.js under the temporary civicconnect-temp-provisioner user (TD-004; DEC-003 v0.4 step 5): on the test cluster on 2026-10-14 and on the staging cluster on 2026-10-15.</t>
+  </si>
+  <si>
+    <t>docs/evidence/M3-indexes/index_duplicate_refusal_test_2026-10-14.txt, L3: a duplicate (requestId, requestVersion) refused with 11000 naming the index. On staging the index is listed as present and unique: docs/evidence/M3-indexes/index_provisioning_staging_run1.txt and _run2.txt (PR #111): RESULT PASS 21 of 21 on the staging cluster, 2026-10-15. Duplicate refusal itself was exercised on the test cluster only.</t>
+  </si>
+  <si>
+    <t>The unique index email_1 was built by scripts/atlas/provision-indexes.js under the temporary civicconnect-temp-provisioner user (TD-004; DEC-003 v0.4 step 5): on the test cluster on 2026-10-14 and on the staging cluster on 2026-10-15. Whether scripts/admin/create-user.js should also check for an existing email before inserting is still to be decided.</t>
+  </si>
+  <si>
+    <t>docs/evidence/M3-indexes/index_duplicate_refusal_test_2026-10-14.txt, L4: a duplicate email refused with 11000 naming the index. On staging the index is listed as present and unique: docs/evidence/M3-indexes/index_provisioning_staging_run1.txt and _run2.txt (PR #111): RESULT PASS 21 of 21 on the staging cluster, 2026-10-15. Duplicate refusal itself was exercised on the test cluster only.</t>
+  </si>
+  <si>
+    <t>DEF-020</t>
+  </si>
+  <si>
+    <t>R. van der Merwe, during the staging deploy (fixture attempt 1)</t>
+  </si>
+  <si>
+    <t>MONGODB_URI in /etc/civicconnect/staging.env named no database, so the application connected to the driver's default database, test, instead of civicconnect, from its first start on staging until the service was restarted with the corrected URI at 16:12:28 UTC on 15/10/2026. Found at about 15:27 UTC, when the first fixture run was refused with "not allowed to do action [find] on [test.users]". The connection and the /health ping succeeded throughout, so the step 7 health check (14:19:22 UTC) did not reveal it. src/config.js states that the application "refuses to start on a missing or malformed value rather than falling back to a default", but it checks only that MONGODB_URI is set and has the mongodb scheme, so a URI without a database name passes. Neither DEC-003 nor .env.example says the URI must name the database.</t>
+  </si>
+  <si>
+    <t>Staging configuration (/etc/civicconnect/staging.env); src/config.js; .env.example; DEC-003 v0.4 (Secrets, deployment procedure); NFR-1.6 (/health)</t>
+  </si>
+  <si>
+    <t>While it lasted, the deployed release candidate could not read or write request data on staging: civicconnect-app has no grants on the test database. /health reported the database up, so the deploy's own check could not see the fault. The same mistake in production would leave the service reporting healthy while every data request failed.</t>
+  </si>
+  <si>
+    <t>/civicconnect added to the URI in /etc/civicconnect/staging.env and the service restarted (by 16:12:28 UTC on 15/10/2026). The perf fixture and cleanup scripts now refuse a URI that does not name the civicconnect database (PR #110). Not done: src/config.js and .env.example do not require the database name; that is for a later code change and the next DEC-003 version.</t>
+  </si>
+  <si>
+    <t>PR #111 (deploy record, section 3, Configuration correction); PR #110 (fixture scripts' database guard)</t>
+  </si>
+  <si>
+    <t>After the correction, the NFR-2.4 load run (16:30:21 to 16:41:31 UTC) logged in all 100 fixture users written to civicconnect at 16:25 and passed, and smoke check 1 (17:02:22 UTC) returned /health 200 with release 30ff0c6 (docs/evidence/M3_Staging_Deploy_v3.0-M3-rc.md, sections 8 and 9; PR #111).</t>
+  </si>
+  <si>
+    <t>Closed on staging. Residual: the application does not refuse a MONGODB_URI without a database name, and /health does not report which database it uses, so the same mistake on another environment would again pass the health check.</t>
+  </si>
+  <si>
+    <t>Robert</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1022,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:O29"/>
+  <dimension ref="B1:O30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -1024,7 +1048,7 @@
     </row>
     <row r="2" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.3">
@@ -1338,7 +1362,7 @@
         <v>33</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>70</v>
@@ -1713,19 +1737,19 @@
         <v>27</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="N24" s="5" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="O24" s="5" t="s">
         <v>33</v>
@@ -1758,19 +1782,19 @@
         <v>27</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="N25" s="5" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="O25" s="5" t="s">
         <v>33</v>
@@ -1848,19 +1872,19 @@
         <v>27</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="N27" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="O27" s="6" t="s">
         <v>33</v>
@@ -1913,26 +1937,26 @@
     </row>
     <row r="29" spans="2:15" ht="174" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="C29" s="4">
         <f>DATE(2026,10,15)</f>
         <v>46310</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>25</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="I29" s="6" t="s">
         <v>65</v>
@@ -1941,23 +1965,68 @@
         <v>66</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="L29" s="6" t="s">
         <v>67</v>
       </c>
       <c r="M29" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="N29" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="O29" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="2:15" ht="211.2" x14ac:dyDescent="0.3">
+      <c r="B30" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="N29" s="6" t="s">
+      <c r="C30" s="4">
+        <f>DATE(2026,10,15)</f>
+        <v>46310</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="O29" s="6" t="s">
-        <v>33</v>
+      <c r="E30" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="M30" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="N30" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="O30" s="6" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B10:O29" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="B10:O30" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>